<commit_message>
fix(gantt): Correct Excel Gantt stacked bar offsets, date axis bounds, and category labels
</commit_message>
<xml_diff>
--- a/project_management/Planning_WMS.xlsx
+++ b/project_management/Planning_WMS.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -130,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -144,6 +146,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -152,6 +157,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -275,6 +283,32 @@
           <order val="0"/>
           <tx>
             <strRef>
+              <f>'WMS Agile Project Schedule'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'WMS Agile Project Schedule'!$A$5:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'WMS Agile Project Schedule'!$B$5:$B$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
               <f>'WMS Agile Project Schedule'!C4</f>
             </strRef>
           </tx>
@@ -306,9 +340,12 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="46292"/>
+          <min val="46204"/>
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <numFmt formatCode="yyyy-mm-dd" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -323,6 +360,7 @@
         <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -341,7 +379,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="5760000"/>
+    <ext cx="10080000" cy="6480000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -653,7 +691,7 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -661,21 +699,21 @@
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Warehouse Stock Inventory System - Agile Sprint Planning &amp; Schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
+          <t>Warehouse Stock Inventory System - Agile Sprint Planning &amp; Gantt Schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course: CSE 220 Software Engineering | Team: Ankit Katwal (Lead), Sabrin Manandhar (Scrum Master), Shivam Khadka (DevOps)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
+          <t>Course: CSE 220 Software Engineering | IAU | Team: Ankit Katwal (Lead), Sabrin Manandhar (Scrum Master), Shivam Khadka (DevOps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Task / Story ID &amp; Description</t>
@@ -688,7 +726,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Est. Days</t>
+          <t>Duration (Days)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -723,24 +761,20 @@
           <t>Sprint 1 Planning &amp; Backlog Refinement</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
+      <c r="B5" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="E5" s="5">
+      <c r="D5" s="5" t="n">
+        <v>46205</v>
+      </c>
+      <c r="E5" s="6">
         <f>(D5-B5)+1</f>
         <v/>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -750,75 +784,67 @@
           <t>All Members</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>WMS-01: User Authentication &amp; Role Access</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
+      <c r="B6" s="9" t="n">
+        <v>46206</v>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="E6" s="8">
+      <c r="D6" s="9" t="n">
+        <v>46210</v>
+      </c>
+      <c r="E6" s="10">
         <f>(D6-B6)+1</f>
         <v/>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>2 pts</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Ankit Katwal</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>WMS-02: Incoming Stock Intake &amp; PO Logging</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
+      <c r="B7" s="5" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C7" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="E7" s="5">
+      <c r="D7" s="5" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E7" s="6">
         <f>(D7-B7)+1</f>
         <v/>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>5 pts</t>
         </is>
@@ -828,75 +854,67 @@
           <t>Shivam Khadka</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>WMS-03: Handheld Barcode &amp; QR Scanner</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
+      <c r="B8" s="9" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C8" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="E8" s="8">
+      <c r="D8" s="9" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E8" s="10">
         <f>(D8-B8)+1</f>
         <v/>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>3 pts</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Ankit Katwal</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>WMS-04: Real-Time Stock Availability Check</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
+      <c r="B9" s="5" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="E9" s="5">
+      <c r="D9" s="5" t="n">
+        <v>46228</v>
+      </c>
+      <c r="E9" s="6">
         <f>(D9-B9)+1</f>
         <v/>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>3 pts</t>
         </is>
@@ -906,46 +924,42 @@
           <t>Sabrin Manandhar</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Sprint 1 QA Review &amp; Retrospective</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n">
+      <c r="B10" s="9" t="n">
+        <v>46229</v>
+      </c>
+      <c r="C10" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="E10" s="8">
+      <c r="D10" s="9" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E10" s="10">
         <f>(D10-B10)+1</f>
         <v/>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>All Members</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
@@ -957,24 +971,20 @@
           <t>Sprint 2 Planning &amp; Backlog Refinement</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
+      <c r="B11" s="5" t="n">
+        <v>46231</v>
+      </c>
+      <c r="C11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="E11" s="5">
+      <c r="D11" s="5" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E11" s="6">
         <f>(D11-B11)+1</f>
         <v/>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -984,75 +994,67 @@
           <t>All Members</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>WMS-05: Low-Stock Watchlist &amp; Threshold Alerts</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n">
+      <c r="B12" s="9" t="n">
+        <v>46232</v>
+      </c>
+      <c r="C12" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="E12" s="8">
+      <c r="D12" s="9" t="n">
+        <v>46237</v>
+      </c>
+      <c r="E12" s="10">
         <f>(D12-B12)+1</f>
         <v/>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>3 pts</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Sabrin Manandhar</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>WMS-06: Urgent Order Priority Tagging</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
+      <c r="B13" s="5" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="E13" s="5">
+      <c r="D13" s="5" t="n">
+        <v>46241</v>
+      </c>
+      <c r="E13" s="6">
         <f>(D13-B13)+1</f>
         <v/>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>2 pts</t>
         </is>
@@ -1062,46 +1064,42 @@
           <t>Ankit Katwal</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>WMS-07: Atomic Stock Reservation &amp; Locking</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
+      <c r="B14" s="9" t="n">
+        <v>46242</v>
+      </c>
+      <c r="C14" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="E14" s="8">
+      <c r="D14" s="9" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E14" s="10">
         <f>(D14-B14)+1</f>
         <v/>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>5 pts</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Shivam Khadka</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
@@ -1113,24 +1111,20 @@
           <t>Sprint 2 QA Review &amp; Retrospective</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
+      <c r="B15" s="5" t="n">
+        <v>46249</v>
+      </c>
+      <c r="C15" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="E15" s="5">
+      <c r="D15" s="5" t="n">
+        <v>46250</v>
+      </c>
+      <c r="E15" s="6">
         <f>(D15-B15)+1</f>
         <v/>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1140,75 +1134,67 @@
           <t>All Members</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Sprint 3 Planning &amp; Backlog Refinement</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
+      <c r="B16" s="9" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="E16" s="8">
+      <c r="D16" s="9" t="n">
+        <v>46251</v>
+      </c>
+      <c r="E16" s="10">
         <f>(D16-B16)+1</f>
         <v/>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>All Members</t>
         </is>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>WMS-08: Supplier Replenishment PO Transmission</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
+      <c r="B17" s="5" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C17" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="E17" s="5">
+      <c r="D17" s="5" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E17" s="6">
         <f>(D17-B17)+1</f>
         <v/>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>5 pts</t>
         </is>
@@ -1218,75 +1204,67 @@
           <t>Shivam Khadka</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>WMS-09: Itemized Dispatch Note Generation</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="n">
+      <c r="B18" s="9" t="n">
+        <v>46259</v>
+      </c>
+      <c r="C18" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="E18" s="8">
+      <c r="D18" s="9" t="n">
+        <v>46263</v>
+      </c>
+      <c r="E18" s="10">
         <f>(D18-B18)+1</f>
         <v/>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>3 pts</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>Sabrin Manandhar</t>
         </is>
       </c>
-      <c r="H18" s="12" t="inlineStr">
+      <c r="H18" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>WMS-10: Immutable Audit Transaction Ledger</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
+      <c r="B19" s="5" t="n">
+        <v>46264</v>
+      </c>
+      <c r="C19" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E19" s="5">
+      <c r="D19" s="5" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E19" s="6">
         <f>(D19-B19)+1</f>
         <v/>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>3 pts</t>
         </is>
@@ -1296,46 +1274,42 @@
           <t>Ankit Katwal</t>
         </is>
       </c>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="H19" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Sprint 3 QA Review &amp; Retrospective</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
+      <c r="B20" s="9" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C20" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="E20" s="8">
+      <c r="D20" s="9" t="n">
+        <v>46271</v>
+      </c>
+      <c r="E20" s="10">
         <f>(D20-B20)+1</f>
         <v/>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>All Members</t>
         </is>
       </c>
-      <c r="H20" s="12" t="inlineStr">
+      <c r="H20" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -1347,24 +1321,20 @@
           <t>Sprint 4 Planning &amp; Test Matrix Alignment</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
+      <c r="B21" s="5" t="n">
+        <v>46272</v>
+      </c>
+      <c r="C21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="E21" s="5">
+      <c r="D21" s="5" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E21" s="6">
         <f>(D21-B21)+1</f>
         <v/>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1374,46 +1344,42 @@
           <t>All Members</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
+      <c r="H21" s="15" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Master Test Matrix QA (40 Test Cases)</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
+      <c r="B22" s="9" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C22" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="E22" s="8">
+      <c r="D22" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E22" s="10">
         <f>(D22-B22)+1</f>
         <v/>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
         <is>
           <t>40 Cases</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>Sabrin Manandhar</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="H22" s="15" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
@@ -1425,24 +1391,20 @@
           <t>GitHub Repository Branch &amp; Pull Request Merge</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="n">
+      <c r="B23" s="5" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C23" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="E23" s="5">
+      <c r="D23" s="5" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E23" s="6">
         <f>(D23-B23)+1</f>
         <v/>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>CI/CD</t>
         </is>
@@ -1452,46 +1414,42 @@
           <t>Shivam Khadka</t>
         </is>
       </c>
-      <c r="H23" s="13" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Final Project Report Finalization &amp; APA 7 Audit</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n">
+      <c r="B24" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C24" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E24" s="8">
+      <c r="D24" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E24" s="10">
         <f>(D24-B24)+1</f>
         <v/>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>All Members</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr">
+      <c r="H24" s="15" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
@@ -1503,24 +1461,20 @@
           <t>Final Sprint Review &amp; Deployment Sign-Off</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="n">
+      <c r="B25" s="5" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C25" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E25" s="5">
+      <c r="D25" s="5" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E25" s="6">
         <f>(D25-B25)+1</f>
         <v/>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1530,7 +1484,7 @@
           <t>All Members</t>
         </is>
       </c>
-      <c r="H25" s="13" t="inlineStr">
+      <c r="H25" s="15" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>

</xml_diff>

<commit_message>
fix(final-audit): Synchronize exact 8-week schedule, clean UML models, and APA 7th report
</commit_message>
<xml_diff>
--- a/project_management/Planning_WMS.xlsx
+++ b/project_management/Planning_WMS.xlsx
@@ -268,7 +268,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Warehouse Stock Inventory System - Agile Sprint Gantt Schedule</a:t>
+              <a:t>Warehouse Stock Inventory System - 8-Week Agile Sprint Schedule</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -340,7 +340,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="46292"/>
+          <max val="46261"/>
           <min val="46204"/>
         </scaling>
         <axPos val="l"/>
@@ -702,7 +702,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Warehouse Stock Inventory System - Agile Sprint Planning &amp; Gantt Schedule</t>
+          <t>Warehouse Stock Inventory System - 8-Week Agile Project Schedule &amp; Gantt</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Sprint 1 Planning &amp; Backlog Refinement</t>
+          <t>Sprint 1 Kickoff &amp; Requirements Elicitation</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -800,10 +800,10 @@
         <v>46206</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="E6" s="10">
         <f>(D6-B6)+1</f>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46211</v>
+        <v>46208</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>46217</v>
+        <v>46213</v>
       </c>
       <c r="E7" s="6">
         <f>(D7-B7)+1</f>
@@ -867,13 +867,13 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>46218</v>
+        <v>46211</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>46223</v>
+        <v>46215</v>
       </c>
       <c r="E8" s="10">
         <f>(D8-B8)+1</f>
@@ -902,13 +902,13 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>46224</v>
+        <v>46212</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>5</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>46228</v>
+        <v>46216</v>
       </c>
       <c r="E9" s="6">
         <f>(D9-B9)+1</f>
@@ -937,13 +937,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>46229</v>
+        <v>46216</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>2</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>46230</v>
+        <v>46217</v>
       </c>
       <c r="E10" s="10">
         <f>(D10-B10)+1</f>
@@ -972,13 +972,13 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>46231</v>
+        <v>46218</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>46231</v>
+        <v>46218</v>
       </c>
       <c r="E11" s="6">
         <f>(D11-B11)+1</f>
@@ -1007,13 +1007,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>46232</v>
+        <v>46219</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>46237</v>
+        <v>46223</v>
       </c>
       <c r="E12" s="10">
         <f>(D12-B12)+1</f>
@@ -1042,13 +1042,13 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>46238</v>
+        <v>46221</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>46241</v>
+        <v>46225</v>
       </c>
       <c r="E13" s="6">
         <f>(D13-B13)+1</f>
@@ -1077,13 +1077,13 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>46242</v>
+        <v>46223</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>7</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>46248</v>
+        <v>46229</v>
       </c>
       <c r="E14" s="10">
         <f>(D14-B14)+1</f>
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>46249</v>
+        <v>46230</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>46250</v>
+        <v>46231</v>
       </c>
       <c r="E15" s="6">
         <f>(D15-B15)+1</f>
@@ -1147,13 +1147,13 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>46251</v>
+        <v>46232</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>46251</v>
+        <v>46232</v>
       </c>
       <c r="E16" s="10">
         <f>(D16-B16)+1</f>
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>46252</v>
+        <v>46233</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>7</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>46258</v>
+        <v>46239</v>
       </c>
       <c r="E17" s="6">
         <f>(D17-B17)+1</f>
@@ -1217,13 +1217,13 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>46259</v>
+        <v>46237</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>46263</v>
+        <v>46242</v>
       </c>
       <c r="E18" s="10">
         <f>(D18-B18)+1</f>
@@ -1252,13 +1252,13 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>46264</v>
+        <v>46238</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>46269</v>
+        <v>46243</v>
       </c>
       <c r="E19" s="6">
         <f>(D19-B19)+1</f>
@@ -1287,13 +1287,13 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>46270</v>
+        <v>46244</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>2</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>46271</v>
+        <v>46245</v>
       </c>
       <c r="E20" s="10">
         <f>(D20-B20)+1</f>
@@ -1322,13 +1322,13 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>46272</v>
+        <v>46246</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>46272</v>
+        <v>46246</v>
       </c>
       <c r="E21" s="6">
         <f>(D21-B21)+1</f>
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>46273</v>
+        <v>46247</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>46279</v>
+        <v>46252</v>
       </c>
       <c r="E22" s="10">
         <f>(D22-B22)+1</f>
@@ -1388,17 +1388,17 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>GitHub Repository Branch &amp; Pull Request Merge</t>
+          <t>GitHub Repo Branch &amp; Pull Request Integration</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>46280</v>
+        <v>46251</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>46283</v>
+        <v>46255</v>
       </c>
       <c r="E23" s="6">
         <f>(D23-B23)+1</f>
@@ -1427,13 +1427,13 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>46284</v>
+        <v>46253</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>46288</v>
+        <v>46258</v>
       </c>
       <c r="E24" s="10">
         <f>(D24-B24)+1</f>
@@ -1462,13 +1462,13 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>46289</v>
+        <v>46259</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>46289</v>
+        <v>46259</v>
       </c>
       <c r="E25" s="6">
         <f>(D25-B25)+1</f>

</xml_diff>